<commit_message>
Slicing TDDUIBundle entry 1a3b7c9b9e2178ed40a3aa0be0ada254b29744db
</commit_message>
<xml_diff>
--- a/ig/specifications_techniques/StructureDefinition-tddui-documentreference.xlsx
+++ b/ig/specifications_techniques/StructureDefinition-tddui-documentreference.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.2.0</t>
+    <t>1.0.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-10-02T08:19:52+00:00</t>
+    <t>2023-10-02T10:10:17+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>